<commit_message>
Quitar ingreso de codigo otp
</commit_message>
<xml_diff>
--- a/src/equipos/equipos.xlsx
+++ b/src/equipos/equipos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,19 +498,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479349</t>
+          <t xml:space="preserve"> 57101602404485988</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403764682</t>
+          <t xml:space="preserve"> 352855403634208</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D2" t="n">
-        <v>3103962743</v>
+        <v>3217671098</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -525,19 +525,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479350</t>
+          <t xml:space="preserve"> 57101602404485995</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403768410</t>
+          <t xml:space="preserve"> 352855403646806</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D3" t="n">
-        <v>3103970793</v>
+        <v>3217672936</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -552,19 +552,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479352</t>
+          <t xml:space="preserve"> 57101602404485996</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403768675</t>
+          <t xml:space="preserve"> 352855403654446</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D4" t="n">
-        <v>3103512281</v>
+        <v>3217676235</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -579,19 +579,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479353</t>
+          <t xml:space="preserve"> 57101602404486000</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403769640</t>
+          <t xml:space="preserve"> 352855403658033</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D5" t="n">
-        <v>3103518581</v>
+        <v>3217683800</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -606,19 +606,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479362</t>
+          <t xml:space="preserve"> 57101602404486003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403765853</t>
+          <t xml:space="preserve"> 352855403658538</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D6" t="n">
-        <v>3103503570</v>
+        <v>3217687642</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -633,18 +633,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479364</t>
+          <t xml:space="preserve"> 57101602404486005</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403831457</t>
+          <t xml:space="preserve"> 352855403658793</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3217692653</v>
+      </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -658,21 +660,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479369</t>
+          <t xml:space="preserve"> 57101602404486006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403843254</t>
+          <t xml:space="preserve"> 352855403659270</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>3103578810</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3217693973</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -687,23 +687,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479375</t>
+          <t xml:space="preserve"> 57101602404486009</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403853162</t>
+          <t xml:space="preserve"> 352855403659734</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3113145589</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>La activación no puede continuar por las siguientes razones:</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -716,21 +720,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479376</t>
+          <t xml:space="preserve"> 57101602404486010</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403881643</t>
+          <t xml:space="preserve"> 352855403659940</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>3114113274</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3217704043</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -745,21 +747,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479378</t>
+          <t xml:space="preserve"> 57101602404486011</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403882369</t>
+          <t xml:space="preserve"> 352855403660328</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>3114126495</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3217710170</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -774,21 +774,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479385</t>
+          <t xml:space="preserve"> 57101602404486012</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403882559</t>
+          <t xml:space="preserve"> 352855403661359</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>3113167861</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3217639789</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -803,21 +801,19 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479386</t>
+          <t xml:space="preserve"> 57101602404486013</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403883102</t>
+          <t xml:space="preserve"> 352855403661714</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>3113161375</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3217643612</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -832,21 +828,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479394</t>
+          <t xml:space="preserve"> 57101602404486014</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404340839</t>
+          <t xml:space="preserve"> 352855403663314</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>3114134640</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3217650045</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -861,21 +855,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479397</t>
+          <t xml:space="preserve"> 57101602404486015</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404344526</t>
+          <t xml:space="preserve"> 352855403664270</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>3113188359</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3217656296</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -890,21 +882,19 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479406</t>
+          <t xml:space="preserve"> 57101602404486016</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404350341</t>
+          <t xml:space="preserve"> 352855403664502</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>3113185861</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3217657624</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -919,21 +909,19 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479407</t>
+          <t xml:space="preserve"> 57101602404486017</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404357346</t>
+          <t xml:space="preserve"> 352855403664684</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>3114147325</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3217662625</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -948,21 +936,19 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479412</t>
+          <t xml:space="preserve"> 57101602404486018</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404359854</t>
+          <t xml:space="preserve"> 352855403664866</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>3113191834</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3217665169</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -977,21 +963,19 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479413</t>
+          <t xml:space="preserve"> 57101602404486019</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404371230</t>
+          <t xml:space="preserve"> 352855403666374</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>3113012448</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3217672017</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1006,21 +990,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479416</t>
+          <t xml:space="preserve"> 57101602404486020</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403764476</t>
+          <t xml:space="preserve"> 352855403666671</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>3113041024</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3217674067</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1035,21 +1017,19 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479419</t>
+          <t xml:space="preserve"> 57101602404486022</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403765598</t>
+          <t xml:space="preserve"> 352855403667000</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>3113023662</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3217678853</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1064,21 +1044,19 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479420</t>
+          <t xml:space="preserve"> 57101602404486023</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403764716</t>
+          <t xml:space="preserve"> 352855403668040</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>3113043150</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3217685173</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1093,21 +1071,19 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479421</t>
+          <t xml:space="preserve"> 57101602404486024</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403768568</t>
+          <t xml:space="preserve"> 352855403668677</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>3114014792</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3217687667</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1122,20 +1098,20 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479422</t>
+          <t xml:space="preserve"> 57101602404486025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403768691</t>
+          <t xml:space="preserve"> 352855403668784</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3114050303</t>
+          <t>3218456792</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -1151,21 +1127,19 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479423</t>
+          <t xml:space="preserve"> 57101602404486030</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403769988</t>
+          <t xml:space="preserve"> 352855403669014</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>3113074622</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3217696570</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1180,21 +1154,19 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479425</t>
+          <t xml:space="preserve"> 57101602404486031</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403768188</t>
+          <t xml:space="preserve"> 352855403669063</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>3114029099</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3217713018</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1209,21 +1181,19 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479429</t>
+          <t xml:space="preserve"> 57101602404486032</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404340888</t>
+          <t xml:space="preserve"> 352855403669253</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>3113066238</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3217643689</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1238,21 +1208,19 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479430</t>
+          <t xml:space="preserve"> 57101602404486033</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404345978</t>
+          <t xml:space="preserve"> 352855403669469</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>3113035184</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3217648711</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1267,21 +1235,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479431</t>
+          <t xml:space="preserve"> 57101602404486035</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404351992</t>
+          <t xml:space="preserve"> 352855403669543</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>3113084926</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3217653895</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1296,21 +1262,19 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479432</t>
+          <t xml:space="preserve"> 57101602404486036</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404357379</t>
+          <t xml:space="preserve"> 352855403669675</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>3113089092</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3217658973</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
@@ -1325,21 +1289,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479433</t>
+          <t xml:space="preserve"> 57101602404486037</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404369457</t>
+          <t xml:space="preserve"> 352855403669782</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>3113093182</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3217662743</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
@@ -1354,21 +1316,19 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479434</t>
+          <t xml:space="preserve"> 57101602404486038</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855404371446</t>
+          <t xml:space="preserve"> 352855403637649</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>3113202807</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3217670489</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
@@ -1383,21 +1343,19 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479435</t>
+          <t xml:space="preserve"> 57101602404486040</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403831788</t>
+          <t xml:space="preserve"> 352855403647895</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>3113234088</t>
-        </is>
+        <v>1036962271</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3217673059</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
@@ -1412,20 +1370,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479436</t>
+          <t xml:space="preserve"> 57101602404486041</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403847099</t>
+          <t xml:space="preserve"> 352855403657100</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3113235721</t>
+          <t>3218457969</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1441,20 +1399,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479437</t>
+          <t xml:space="preserve"> 57101602404486042</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403859490</t>
+          <t xml:space="preserve"> 352855403658116</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3113099808</t>
+          <t>3218461597</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1470,20 +1428,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479442</t>
+          <t xml:space="preserve"> 57101602404486043</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403882229</t>
+          <t xml:space="preserve"> 352855403658579</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3114068757</t>
+          <t>3218464082</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1499,20 +1457,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479444</t>
+          <t xml:space="preserve"> 57101602404486045</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403882419</t>
+          <t xml:space="preserve"> 352855403658819</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3114061954</t>
+          <t>3218506271</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1528,20 +1486,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479451</t>
+          <t xml:space="preserve"> 57101602404486046</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403882567</t>
+          <t xml:space="preserve"> 352855403659296</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3113216163</t>
+          <t>3218469940</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1557,20 +1515,20 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479454</t>
+          <t xml:space="preserve"> 57101602404486049</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403883268</t>
+          <t xml:space="preserve"> 352855403659767</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1017173051</v>
+        <v>1036962271</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3113217307</t>
+          <t>3218472507</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -1586,18 +1544,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479455</t>
+          <t xml:space="preserve"> 57101602404486051</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403733554</t>
+          <t xml:space="preserve"> 352855403660187</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D40" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>3218481300</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
@@ -1611,18 +1573,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479456</t>
+          <t xml:space="preserve"> 57101602404466055</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403731814</t>
+          <t xml:space="preserve"> 352855403660666</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D41" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3218486390</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
@@ -1636,18 +1602,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479459</t>
+          <t xml:space="preserve"> 57101602404466057</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403791727</t>
+          <t xml:space="preserve"> 352855403661557</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D42" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>3218491450</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
@@ -1661,18 +1631,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479460</t>
+          <t xml:space="preserve"> 57101602404466059</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403973655</t>
+          <t xml:space="preserve"> 352855403661961</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D43" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>3218493970</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
@@ -1686,18 +1660,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479461</t>
+          <t xml:space="preserve"> 57101602404466065</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403977904</t>
+          <t xml:space="preserve"> 352855403663645</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D44" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>3218417906</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
@@ -1711,18 +1689,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479463</t>
+          <t xml:space="preserve"> 57101602404466071</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352010502593190</t>
+          <t xml:space="preserve"> 352855403664361</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D45" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3218419231</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
@@ -1736,18 +1718,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479465</t>
+          <t xml:space="preserve"> 57101602404466072</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 868820084422981</t>
+          <t xml:space="preserve"> 352855403664544</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D46" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>3218424227</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
@@ -1761,18 +1747,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479468</t>
+          <t xml:space="preserve"> 57101602404466073</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 868915070770847</t>
+          <t xml:space="preserve"> 352855403664726</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D47" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>3218426824</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
@@ -1786,18 +1776,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479470</t>
+          <t xml:space="preserve"> 57101602404466074</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 868667076397915</t>
+          <t xml:space="preserve"> 352855403665103</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D48" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>3218443107</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
@@ -1811,18 +1805,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479472</t>
+          <t xml:space="preserve"> 57101602404466079</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354424869141337</t>
+          <t xml:space="preserve"> 352855403666416</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D49" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>3218449412</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
@@ -1836,18 +1834,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479474</t>
+          <t xml:space="preserve"> 57101602404466085</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 861819074754228</t>
+          <t xml:space="preserve"> 352855403666820</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D50" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>3218496986</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
@@ -1861,18 +1863,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702502393035</t>
+          <t xml:space="preserve"> 57101602404466086</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 863914082023704</t>
+          <t xml:space="preserve"> 352855403667075</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D51" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>3218499545</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
@@ -1886,18 +1892,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702409500856</t>
+          <t xml:space="preserve"> 57101602404466088</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 866501073894727</t>
+          <t xml:space="preserve"> 352855403668362</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D52" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>3218503327</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
@@ -1911,18 +1921,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702606366019</t>
+          <t xml:space="preserve"> 57101602404466089</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 356305718732830</t>
+          <t xml:space="preserve"> 352855403668693</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D53" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3218452126</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
@@ -1936,18 +1950,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404479273</t>
+          <t xml:space="preserve"> 57101602404466092</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 352855403773139</t>
+          <t xml:space="preserve"> 352855403668800</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1017173051</v>
-      </c>
-      <c r="D54" t="inlineStr"/>
+        <v>1036962271</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3218453291</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
@@ -1958,6 +1976,1679 @@
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466093</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669022</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>3218455609</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466096</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669071</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>3218459171</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466100</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669329</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>3218461676</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466101</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669485</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>3218464152</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466102</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669584</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>3218464213</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466103</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669709</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>3218506281</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466106</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403670053</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>3218507569</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466107</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403642730</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3218467490</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466108</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403649131</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3218472538</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466110</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403657225</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>3218473826</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466117</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403658439</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>3218477583</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466119</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403658611</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>3218754748</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466124</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403659064</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466126</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403659320</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466129</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403659825</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466130</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403660229</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466131</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403660799</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466132</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403661623</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466133</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403662449</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466134</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403663710</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466135</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664395</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466136</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664569</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466141</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664759</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466145</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403665616</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466146</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403666440</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466148</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403666895</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466155</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403667208</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466156</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403668529</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466165</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403668735</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466167</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403668834</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466168</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669048</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466170</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669097</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466172</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669386</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466175</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669501</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466179</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669626</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466182</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669717</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466183</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403646483</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466186</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403652903</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466188</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403657720</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466191</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403658504</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466193</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403658710</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466195</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403659130</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466201</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403659676</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466205</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403659908</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466207</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403660260</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466211</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403661177</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466214</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403661664</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466222</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403663074</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466223</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664213</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466228</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664411</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466230</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664593</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466233</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403664791</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466237</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403665723</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466239</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403666564</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466241</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403666929</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466249</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403668032</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466252</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403668602</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466257</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403668776</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466259</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669006</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466262</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669055</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466264</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669188</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466265</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669410</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466266</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669527</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466268</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669659</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404466269</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 352855403669733</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix equipos: actualizar contador de fila
</commit_message>
<xml_diff>
--- a/src/equipos/equipos.xlsx
+++ b/src/equipos/equipos.xlsx
@@ -2338,7 +2338,11 @@
       <c r="C67" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>3226227347</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
@@ -2363,7 +2367,11 @@
       <c r="C68" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>3225224268</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
@@ -2388,7 +2396,11 @@
       <c r="C69" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>3226254940</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
@@ -2413,7 +2425,11 @@
       <c r="C70" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>3225213844</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
@@ -2438,7 +2454,11 @@
       <c r="C71" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>3226283905</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
@@ -2463,7 +2483,11 @@
       <c r="C72" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>3225190358</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
@@ -2488,7 +2512,11 @@
       <c r="C73" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>3226245224</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
@@ -2513,7 +2541,11 @@
       <c r="C74" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>3225186717</t>
+        </is>
+      </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
@@ -2538,7 +2570,11 @@
       <c r="C75" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>3226249087</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
@@ -2563,7 +2599,11 @@
       <c r="C76" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>3225160596</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
@@ -2589,7 +2629,11 @@
         <v>1036962271</v>
       </c>
       <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>La activación no puede continuar por las siguientes razones:</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
@@ -2613,7 +2657,11 @@
       <c r="C78" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>3225178104</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
@@ -2638,7 +2686,11 @@
       <c r="C79" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>3225186956</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
@@ -2663,7 +2715,11 @@
       <c r="C80" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>3225160815</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
@@ -2688,7 +2744,11 @@
       <c r="C81" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>3225203983</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>

</xml_diff>

<commit_message>
Forzar error cuando login falla por usuario en el sistema
</commit_message>
<xml_diff>
--- a/src/equipos/equipos.xlsx
+++ b/src/equipos/equipos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,27 +498,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473436</t>
+          <t xml:space="preserve"> 57101602404474848</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 350357335251567</t>
+          <t xml:space="preserve"> 866567079343001</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>9918INV-021. El IMEI: "350357335251567", no pertenece al distribuidor</t>
-        </is>
-      </c>
+      <c r="D2" t="n">
+        <v>3227803460</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -531,27 +525,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473437</t>
+          <t xml:space="preserve"> 57101602404474849</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 350715442088984</t>
+          <t xml:space="preserve"> 860688079277449</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>9918INV-021. El IMEI: "350715442088984", no pertenece al distribuidor</t>
-        </is>
-      </c>
+      <c r="D3" t="n">
+        <v>3227848806</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -564,21 +552,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473438</t>
+          <t xml:space="preserve"> 57101602404474850</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351001190071590</t>
+          <t xml:space="preserve"> 860688079848843</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>3232119670</t>
-        </is>
+      <c r="D4" t="n">
+        <v>3227896998</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -593,21 +579,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473439</t>
+          <t xml:space="preserve"> 57101602404474851</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351001190078306</t>
+          <t xml:space="preserve"> 860688073778285</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>3232124653</t>
-        </is>
+      <c r="D5" t="n">
+        <v>3227887525</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -622,21 +606,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473441</t>
+          <t xml:space="preserve"> 57101602404474852</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351001190094436</t>
+          <t xml:space="preserve"> 860688071558986</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>3232127172</t>
-        </is>
+      <c r="D6" t="n">
+        <v>3227907681</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -651,21 +633,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473442</t>
+          <t xml:space="preserve"> 57101602404474853</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351001190101538</t>
+          <t xml:space="preserve"> 860688073852247</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>3232132147</t>
-        </is>
+      <c r="D7" t="n">
+        <v>3227896602</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -680,21 +660,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473443</t>
+          <t xml:space="preserve"> 57101602404474854</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351001190137060</t>
+          <t xml:space="preserve"> 863391072691925</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>3232134644</t>
-        </is>
+      <c r="D8" t="n">
+        <v>3227901627</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -709,21 +687,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473444</t>
+          <t xml:space="preserve"> 57101602404474857</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351001190138837</t>
+          <t xml:space="preserve"> 860688073757081</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>3232137186</t>
-        </is>
+      <c r="D9" t="n">
+        <v>3227935124</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -738,21 +714,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473448</t>
+          <t xml:space="preserve"> 57101602404474860</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351113352148486</t>
+          <t xml:space="preserve"> 863391073203100</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>3232139630</t>
-        </is>
+      <c r="D10" t="n">
+        <v>3227864194</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -767,21 +741,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473449</t>
+          <t xml:space="preserve"> 57101602404474869</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351113354744720</t>
+          <t xml:space="preserve"> 860688071867965</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>3232142114</t>
-        </is>
+      <c r="D11" t="n">
+        <v>3228003148</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -796,27 +768,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473451</t>
+          <t xml:space="preserve"> 57101602404474870</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351165146777269</t>
+          <t xml:space="preserve"> 860688073820004</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>9918INV-021. El IMEI: "351165146777269", no pertenece al distribuidor</t>
-        </is>
-      </c>
+      <c r="D12" t="n">
+        <v>3227956733</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -829,27 +795,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473452</t>
+          <t xml:space="preserve"> 57101602404474871</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 351517238648479</t>
+          <t xml:space="preserve"> 860688073882467</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>9918INV-021. El IMEI: "351517238648479", no pertenece al distribuidor</t>
-        </is>
-      </c>
+      <c r="D13" t="n">
+        <v>3227970540</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -862,21 +822,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473454</t>
+          <t xml:space="preserve"> 57101602404474872</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353167580035889</t>
+          <t xml:space="preserve"> 867469072921728</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>3232147174</t>
-        </is>
+      <c r="D14" t="n">
+        <v>3228010403</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -891,21 +849,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473460</t>
+          <t xml:space="preserve"> 57101602404474874</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353167580155182</t>
+          <t xml:space="preserve"> 863391072081986</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>3232154728</t>
-        </is>
+      <c r="D15" t="n">
+        <v>3227940647</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -920,21 +876,19 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473462</t>
+          <t xml:space="preserve"> 57101602404474876</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353270600923637</t>
+          <t xml:space="preserve"> 353270600927919</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>3232159663</t>
-        </is>
+      <c r="D16" t="n">
+        <v>3227943151</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -949,21 +903,19 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473464</t>
+          <t xml:space="preserve"> 57101602404474878</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353270601047477</t>
+          <t xml:space="preserve"> 353270600928263</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>3232160925</t>
-        </is>
+      <c r="D17" t="n">
+        <v>3227941926</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -978,27 +930,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473465</t>
+          <t xml:space="preserve"> 57101602404474882</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353506851314640</t>
+          <t xml:space="preserve"> 353270600928438</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>9918INV-021. El IMEI: "353506851314640", no pertenece al distribuidor</t>
-        </is>
-      </c>
+      <c r="D18" t="n">
+        <v>3227945865</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -1011,21 +957,19 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473466</t>
+          <t xml:space="preserve"> 57101602404474890</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353913340027058</t>
+          <t xml:space="preserve"> 353270600963740</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>3232162218</t>
-        </is>
+      <c r="D19" t="n">
+        <v>3227962058</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1040,21 +984,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473470</t>
+          <t xml:space="preserve"> 57101602404474891</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353913340052890</t>
+          <t xml:space="preserve"> 353270600964359</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>3232163465</t>
-        </is>
+      <c r="D20" t="n">
+        <v>3227967044</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1069,27 +1011,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473472</t>
+          <t xml:space="preserve"> 57101602404474895</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 353922390045472</t>
+          <t xml:space="preserve"> 353270600966289</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>9918INV-021. El IMEI: "353922390045472", no pertenece al distribuidor</t>
-        </is>
-      </c>
+      <c r="D21" t="n">
+        <v>3227973292</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -1102,21 +1038,19 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473475</t>
+          <t xml:space="preserve"> 57101602404474898</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354061764133769</t>
+          <t xml:space="preserve"> 353270600967626</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>3232165924</t>
-        </is>
+      <c r="D22" t="n">
+        <v>3227975858</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1131,21 +1065,19 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473476</t>
+          <t xml:space="preserve"> 57101602404474913</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354061764343384</t>
+          <t xml:space="preserve"> 353270600968079</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>3232167261</t>
-        </is>
+      <c r="D23" t="n">
+        <v>3227975874</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1160,21 +1092,19 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473477</t>
+          <t xml:space="preserve"> 57101602404474915</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354061764365072</t>
+          <t xml:space="preserve"> 353270600969283</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>3232167639</t>
-        </is>
+      <c r="D24" t="n">
+        <v>3227977129</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -1189,21 +1119,19 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473487</t>
+          <t xml:space="preserve"> 57101602404474921</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354549780152227</t>
+          <t xml:space="preserve"> 353270600969705</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>3232167949</t>
-        </is>
+      <c r="D25" t="n">
+        <v>3227979628</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1218,21 +1146,19 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473488</t>
+          <t xml:space="preserve"> 57101602404474923</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354549780172837</t>
+          <t xml:space="preserve"> 353270600971404</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>3232168327</t>
-        </is>
+      <c r="D26" t="n">
+        <v>3227983396</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1247,21 +1173,19 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473492</t>
+          <t xml:space="preserve"> 57101602404474925</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354825494648043</t>
+          <t xml:space="preserve"> 353270600971594</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>3232168356</t>
-        </is>
+      <c r="D27" t="n">
+        <v>3227987106</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1276,21 +1200,19 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473493</t>
+          <t xml:space="preserve"> 57101602404474927</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354825494660261</t>
+          <t xml:space="preserve"> 353270600971974</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>3232190153</t>
-        </is>
+      <c r="D28" t="n">
+        <v>3228017604</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1305,21 +1227,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473494</t>
+          <t xml:space="preserve"> 57101602404474929</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 354825494852314</t>
+          <t xml:space="preserve"> 353270600973038</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>3232190850</t>
-        </is>
+      <c r="D29" t="n">
+        <v>3227997370</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1334,21 +1254,19 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473496</t>
+          <t xml:space="preserve"> 57101602404474930</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 355204630112281</t>
+          <t xml:space="preserve"> 353270600973053</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>3232169103</t>
-        </is>
+      <c r="D30" t="n">
+        <v>3228007386</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
@@ -1363,21 +1281,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473498</t>
+          <t xml:space="preserve"> 57101602404474932</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 355233940074691</t>
+          <t xml:space="preserve"> 353270600973772</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>3232169886</t>
-        </is>
+      <c r="D31" t="n">
+        <v>3227943424</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
@@ -1392,21 +1308,19 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473499</t>
+          <t xml:space="preserve"> 57101602404474939</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 355233940103169</t>
+          <t xml:space="preserve"> 353270600974200</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>3232169935</t>
-        </is>
+      <c r="D32" t="n">
+        <v>3227954703</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
@@ -1421,21 +1335,19 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473500</t>
+          <t xml:space="preserve"> 57101602404474942</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 355748171622462</t>
+          <t xml:space="preserve"> 353270600975140</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>3232170769</t>
-        </is>
+      <c r="D33" t="n">
+        <v>3227978424</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
@@ -1450,12 +1362,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473503</t>
+          <t xml:space="preserve"> 57101602404474943</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 355748174149950</t>
+          <t xml:space="preserve"> 353270600983268</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1463,7 +1375,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3232171699</t>
+          <t>3227962213</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1479,12 +1391,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473504</t>
+          <t xml:space="preserve"> 57101602404474944</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 355924402602991</t>
+          <t xml:space="preserve"> 353270600985040</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1492,7 +1404,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3232172687</t>
+          <t>3227964733</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1508,12 +1420,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473506</t>
+          <t xml:space="preserve"> 57101602404474945</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 356310850578603</t>
+          <t xml:space="preserve"> 353270600985388</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1521,7 +1433,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3232172735</t>
+          <t>3227968490</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1537,12 +1449,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473507</t>
+          <t xml:space="preserve"> 57101602404474946</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 356310851857543</t>
+          <t xml:space="preserve"> 353270600922787</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1550,7 +1462,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3232173813</t>
+          <t>3227970987</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1566,22 +1478,18 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473508</t>
+          <t xml:space="preserve"> 57101602404474947</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 356310852050320</t>
+          <t xml:space="preserve"> 353270600942074</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>3232175003</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
@@ -1595,22 +1503,18 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473510</t>
+          <t xml:space="preserve"> 57101602404474950</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 357837631064734</t>
+          <t xml:space="preserve"> 353270600943460</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>1036962271</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>3232176237</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
@@ -1624,12 +1528,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473514</t>
+          <t xml:space="preserve"> 57101602404474951</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 358082861007959</t>
+          <t xml:space="preserve"> 353270600952560</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1649,12 +1553,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473515</t>
+          <t xml:space="preserve"> 57101602404474952</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 358771350003137</t>
+          <t xml:space="preserve"> 353270600958526</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1674,12 +1578,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473516</t>
+          <t xml:space="preserve"> 57101602404474954</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 358771350198366</t>
+          <t xml:space="preserve"> 353270600984621</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1699,12 +1603,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473520</t>
+          <t xml:space="preserve"> 57101602404474956</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 860688073831902</t>
+          <t xml:space="preserve"> 353270601056437</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1724,12 +1628,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473521</t>
+          <t xml:space="preserve"> 57101602404474957</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 860688074013286</t>
+          <t xml:space="preserve"> 353270600939385</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1749,12 +1653,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473522</t>
+          <t xml:space="preserve"> 57101602404474958</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 860688079818002</t>
+          <t xml:space="preserve"> 353270600964177</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1774,12 +1678,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602404473523</t>
+          <t xml:space="preserve"> 57101602404474959</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 861001071025502</t>
+          <t xml:space="preserve"> 353270600966149</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1799,12 +1703,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602402126717</t>
+          <t xml:space="preserve"> 57101602404474964</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 861108060384376</t>
+          <t xml:space="preserve"> 353270600968269</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1824,12 +1728,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602402126718</t>
+          <t xml:space="preserve"> 57101602404474977</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 861336079452088</t>
+          <t xml:space="preserve"> 353270600974671</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1849,12 +1753,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602402126719</t>
+          <t xml:space="preserve"> 57101602404474979</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 862434060383575</t>
+          <t xml:space="preserve"> 353270601875836</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1874,12 +1778,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602402126724</t>
+          <t xml:space="preserve"> 57101602404474981</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 862434060401096</t>
+          <t xml:space="preserve"> 353270601860507</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1899,12 +1803,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602402126759</t>
+          <t xml:space="preserve"> 57101602404474985</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 863968054410547</t>
+          <t xml:space="preserve"> 353270601755699</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1921,6 +1825,1256 @@
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404474986</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270602057533</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404474995</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270602058374</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404474999</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601905617</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475003</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270602052955</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475008</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601541040</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475010</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601804216</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475015</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601874235</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475016</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601875067</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475018</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601875224</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475020</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601884473</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475021</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601885975</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475025</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601886197</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601886957</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475028</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601886965</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475031</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601886981</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475036</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887070</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475038</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887195</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475041</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887278</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475043</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887427</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475044</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887435</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475049</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887500</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475055</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887534</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475058</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887583</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475070</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601887617</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475071</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601905831</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475072</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601905922</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601906854</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601907522</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475080</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601907944</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475084</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601908439</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475087</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601890215</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475088</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601895008</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475089</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601895396</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475090</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601895594</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475094</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601896360</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475095</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601896584</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475097</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601896733</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475101</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601896741</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475102</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601896766</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475104</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601896774</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475105</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601897103</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475111</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601897160</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475115</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601897525</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475117</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601897582</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475118</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601897640</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475122</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601898051</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475137</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601898069</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475141</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601898135</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475142</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601898192</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101602404475143</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 353270601898234</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1036962271</v>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>